<commit_message>
test(e2e): replace the fixtures with a more thoroughly verified set
Same filenames, better documents, and a verifier that proves more of what
the specs depend on. The set now also carries a genuinely encrypted Office
file (CFB container, ECMA-376 agile encryption) and an opaque unknown-format
blob, which the first pass could not produce.

Regeneration is byte-identical except for the two encrypted files, which
embed fresh salts by design. `--verify` re-checks every claim: the heavy
contract stays above the CDN cutoff, the workbook past the row cap, the scan
has zero extractable text (checked both through the content streams and with
pdftotext), the damaged file still fails to parse, and the encrypted ones
still refuse an empty password.

The preview matrix has to be re-run against these before any of its rows can
be marked covered — see the investigation note in COVERAGE_MAP.md.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/e2e/fixtures/files/registry.xlsx
+++ b/e2e/fixtures/files/registry.xlsx
@@ -8,8 +8,8 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Реестр договоров" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Расчёт" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Примечания" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Сводка" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Черновик" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,13 +19,24 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <b val="1"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="12"/>
     </font>
   </fonts>
   <fills count="2">
@@ -48,8 +59,19 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -415,373 +437,562 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E45"/>
+  <dimension ref="A1:H45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Реестр действующих договоров на 15.01.2026</t>
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Реестр действующих договоров ООО «Ромашка» на 2024 год</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>№</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>Контрагент</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Предмет</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Сумма, ₽</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Предмет договора</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Сроки</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="n"/>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Суммы, BYN</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="n"/>
+      <c r="H3" s="2" t="inlineStr">
         <is>
           <t>Статус</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="n">
-        <v>1</v>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>ООО «Ромашка»</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Сопровождение</t>
-        </is>
-      </c>
-      <c r="D4" t="n">
-        <v>100000</v>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>действует</t>
-        </is>
-      </c>
+      <c r="A4" s="2" t="n"/>
+      <c r="B4" s="2" t="n"/>
+      <c r="C4" s="2" t="n"/>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Начало</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Окончание</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Сумма договора</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Оплачено</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="n"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>ИП Иванов И. И.</t>
+          <t>ООО «Ромашка»</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Поставка</t>
-        </is>
-      </c>
-      <c r="D5" t="n">
-        <v>101250</v>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>продлён</t>
-        </is>
+          <t>Оказание услуг</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>01.01.2024</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>4800</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>ООО «Василёк»</t>
+          <t>ИП Иванов И. И.</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Аренда</t>
-        </is>
-      </c>
-      <c r="D6" t="n">
-        <v>102500</v>
-      </c>
-      <c r="E6" t="inlineStr"/>
+          <t>Поставка оборудования</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>02.02.2024</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>04.12.2024</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>6145</v>
+      </c>
+      <c r="G6" t="n">
+        <v>3072.5</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>На согласовании</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>АО «Одуванчик»</t>
+          <t>ООО «Василёк»</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Консультации</t>
-        </is>
-      </c>
-      <c r="D7" t="n">
-        <v>103750</v>
+          <t>Техническое обслуживание</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>03.03.2024</t>
+        </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>на подписании</t>
+          <t>07.12.2024</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>7490</v>
+      </c>
+      <c r="G7" t="n">
+        <v>5617.5</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Завершён</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>ООО «Клевер»</t>
+          <t>ЗАО «Тестовый Мост»</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Подряд</t>
-        </is>
-      </c>
-      <c r="D8" t="n">
-        <v>105000</v>
+          <t>Аренда помещения</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>04.04.2024</t>
+        </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>закрыт</t>
+          <t>10.12.2024</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>8835</v>
+      </c>
+      <c r="G8" t="n">
+        <v>8835</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Продлён</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>ООО «Ромашка»</t>
+          <t>ООО «ТехноСфера-Плюс»</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Сопровождение</t>
-        </is>
-      </c>
-      <c r="D9" t="n">
-        <v>106250</v>
+          <t>Консультационные услуги</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>05.05.2024</t>
+        </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>действует</t>
+          <t>13.12.2024</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>10180</v>
+      </c>
+      <c r="G9" t="n">
+        <v>2545</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Расторгнут</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>ИП Иванов И. И.</t>
+          <t>ОДО «Северный Ветер»</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Поставка</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>продлён</t>
+          <t>Подряд на монтаж</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>06.06.2024</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>11525</v>
+      </c>
+      <c r="G10" t="n">
+        <v>5762.5</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Действует</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>ООО «Василёк»</t>
+          <t>ООО «Гранит-Строй»</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Аренда</t>
-        </is>
-      </c>
-      <c r="D11" t="n">
-        <v>108750</v>
-      </c>
-      <c r="E11" t="inlineStr"/>
+          <t>Оказание услуг</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>07.07.2024</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>19.12.2024</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
+        <v>12870</v>
+      </c>
+      <c r="G11" t="n">
+        <v>9652.5</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>На согласовании</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>АО «Одуванчик»</t>
+          <t>ООО «Ромашка»</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Консультации</t>
-        </is>
-      </c>
-      <c r="D12" t="n">
-        <v>110000</v>
+          <t>Поставка оборудования</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>08.08.2024</t>
+        </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>на подписании</t>
-        </is>
+          <t>22.12.2024</t>
+        </is>
+      </c>
+      <c r="F12" t="n">
+        <v>12710</v>
+      </c>
+      <c r="G12" t="n">
+        <v>12710</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>ООО «Клевер»</t>
+          <t>ИП Иванов И. И.</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Подряд</t>
-        </is>
-      </c>
-      <c r="D13" t="n">
-        <v>111250</v>
+          <t>Техническое обслуживание</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>09.09.2024</t>
+        </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>закрыт</t>
+          <t>25.12.2024</t>
+        </is>
+      </c>
+      <c r="F13" t="n">
+        <v>14055</v>
+      </c>
+      <c r="G13" t="n">
+        <v>3513.75</v>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Продлён</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>ООО «Ромашка»</t>
+          <t>ООО «Василёк»</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Сопровождение</t>
-        </is>
-      </c>
-      <c r="D14" t="n">
-        <v>112500</v>
+          <t>Аренда помещения</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>10.01.2024</t>
+        </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>действует</t>
+          <t>28.12.2024</t>
+        </is>
+      </c>
+      <c r="F14" t="n">
+        <v>15400</v>
+      </c>
+      <c r="G14" t="n">
+        <v>7700</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Расторгнут</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>ИП Иванов И. И.</t>
+          <t>ЗАО «Тестовый Мост»</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Поставка</t>
-        </is>
-      </c>
-      <c r="D15" t="n">
-        <v>113750</v>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>продлён</t>
+          <t>Консультационные услуги</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>11.02.2024</t>
+        </is>
+      </c>
+      <c r="F15" t="n">
+        <v>16745</v>
+      </c>
+      <c r="G15" t="n">
+        <v>12558.75</v>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Действует</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>ООО «Василёк»</t>
+          <t>ООО «ТехноСфера-Плюс»</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Аренда</t>
-        </is>
-      </c>
-      <c r="D16" t="n">
-        <v>115000</v>
-      </c>
-      <c r="E16" t="inlineStr"/>
+          <t>Подряд на монтаж</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>12.03.2024</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>06.12.2024</t>
+        </is>
+      </c>
+      <c r="F16" t="n">
+        <v>18090</v>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>На согласовании</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>АО «Одуванчик»</t>
+          <t>ОДО «Северный Ветер»</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Консультации</t>
+          <t>Оказание услуг</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>13.04.2024</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>на подписании</t>
+          <t>09.12.2024</t>
+        </is>
+      </c>
+      <c r="F17" t="n">
+        <v>19435</v>
+      </c>
+      <c r="G17" t="n">
+        <v>4858.75</v>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Завершён</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>ООО «Клевер»</t>
+          <t>ООО «Гранит-Строй»</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Подряд</t>
-        </is>
-      </c>
-      <c r="D18" t="n">
-        <v>117500</v>
+          <t>Поставка оборудования</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>14.05.2024</t>
+        </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>закрыт</t>
+          <t>12.12.2024</t>
+        </is>
+      </c>
+      <c r="F18" t="n">
+        <v>20780</v>
+      </c>
+      <c r="G18" t="n">
+        <v>10390</v>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Продлён</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
@@ -790,21 +1001,29 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Сопровождение</t>
-        </is>
-      </c>
-      <c r="D19" t="n">
-        <v>118750</v>
+          <t>Техническое обслуживание</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>15.06.2024</t>
+        </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>действует</t>
-        </is>
+          <t>15.12.2024</t>
+        </is>
+      </c>
+      <c r="F19" t="n">
+        <v>20620</v>
+      </c>
+      <c r="G19" t="n">
+        <v>15465</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
@@ -813,21 +1032,29 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Поставка</t>
-        </is>
-      </c>
-      <c r="D20" t="n">
-        <v>120000</v>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>продлён</t>
+          <t>Аренда помещения</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>16.07.2024</t>
+        </is>
+      </c>
+      <c r="F20" t="n">
+        <v>21965</v>
+      </c>
+      <c r="G20" t="n">
+        <v>21965</v>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Действует</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
@@ -836,510 +1063,846 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Аренда</t>
-        </is>
-      </c>
-      <c r="D21" t="n">
-        <v>121250</v>
-      </c>
-      <c r="E21" t="inlineStr"/>
+          <t>Консультационные услуги</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>17.08.2024</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>21.12.2024</t>
+        </is>
+      </c>
+      <c r="F21" t="n">
+        <v>23310</v>
+      </c>
+      <c r="G21" t="n">
+        <v>5827.5</v>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>На согласовании</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>АО «Одуванчик»</t>
+          <t>ЗАО «Тестовый Мост»</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Консультации</t>
-        </is>
-      </c>
-      <c r="D22" t="n">
-        <v>122500</v>
+          <t>Подряд на монтаж</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>18.09.2024</t>
+        </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>на подписании</t>
+          <t>24.12.2024</t>
+        </is>
+      </c>
+      <c r="F22" t="n">
+        <v>24655</v>
+      </c>
+      <c r="G22" t="n">
+        <v>12327.5</v>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Завершён</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>ООО «Клевер»</t>
+          <t>ООО «ТехноСфера-Плюс»</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Подряд</t>
-        </is>
-      </c>
-      <c r="D23" t="n">
-        <v>123750</v>
+          <t>Оказание услуг</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>19.01.2024</t>
+        </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>закрыт</t>
+          <t>27.12.2024</t>
+        </is>
+      </c>
+      <c r="F23" t="n">
+        <v>26000</v>
+      </c>
+      <c r="G23" t="n">
+        <v>19500</v>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Продлён</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>ООО «Ромашка»</t>
+          <t>ОДО «Северный Ветер»</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Сопровождение</t>
+          <t>Поставка оборудования</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>20.02.2024</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>действует</t>
+          <t>02.12.2024</t>
+        </is>
+      </c>
+      <c r="F24" t="n">
+        <v>27345</v>
+      </c>
+      <c r="G24" t="n">
+        <v>27345</v>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>Расторгнут</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>ИП Иванов И. И.</t>
+          <t>ООО «Гранит-Строй»</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Поставка</t>
-        </is>
-      </c>
-      <c r="D25" t="n">
-        <v>126250</v>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>продлён</t>
+          <t>Техническое обслуживание</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>21.03.2024</t>
+        </is>
+      </c>
+      <c r="F25" t="n">
+        <v>28690</v>
+      </c>
+      <c r="G25" t="n">
+        <v>7172.5</v>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Действует</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>ООО «Василёк»</t>
+          <t>ООО «Ромашка»</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Аренда</t>
-        </is>
-      </c>
-      <c r="D26" t="n">
-        <v>127500</v>
-      </c>
-      <c r="E26" t="inlineStr"/>
+          <t>Аренда помещения</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>22.04.2024</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>08.12.2024</t>
+        </is>
+      </c>
+      <c r="F26" t="n">
+        <v>28530</v>
+      </c>
+      <c r="G26" t="n">
+        <v>14265</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>АО «Одуванчик»</t>
+          <t>ИП Иванов И. И.</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Консультации</t>
-        </is>
-      </c>
-      <c r="D27" t="n">
-        <v>128750</v>
+          <t>Консультационные услуги</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>23.05.2024</t>
+        </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>на подписании</t>
+          <t>11.12.2024</t>
+        </is>
+      </c>
+      <c r="F27" t="n">
+        <v>29875</v>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Завершён</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>ООО «Клевер»</t>
+          <t>ООО «Василёк»</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Подряд</t>
-        </is>
-      </c>
-      <c r="D28" t="n">
-        <v>130000</v>
+          <t>Подряд на монтаж</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>24.06.2024</t>
+        </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>закрыт</t>
+          <t>14.12.2024</t>
+        </is>
+      </c>
+      <c r="F28" t="n">
+        <v>31220</v>
+      </c>
+      <c r="G28" t="n">
+        <v>31220</v>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>Продлён</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>ООО «Ромашка»</t>
+          <t>ЗАО «Тестовый Мост»</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Сопровождение</t>
-        </is>
-      </c>
-      <c r="D29" t="n">
-        <v>131250</v>
+          <t>Оказание услуг</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>25.07.2024</t>
+        </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>действует</t>
+          <t>17.12.2024</t>
+        </is>
+      </c>
+      <c r="F29" t="n">
+        <v>32565</v>
+      </c>
+      <c r="G29" t="n">
+        <v>8141.25</v>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Расторгнут</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>ИП Иванов И. И.</t>
+          <t>ООО «ТехноСфера-Плюс»</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Поставка</t>
-        </is>
-      </c>
-      <c r="D30" t="n">
-        <v>132500</v>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>продлён</t>
+          <t>Поставка оборудования</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>26.08.2024</t>
+        </is>
+      </c>
+      <c r="F30" t="n">
+        <v>33910</v>
+      </c>
+      <c r="G30" t="n">
+        <v>16955</v>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>Действует</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>ООО «Василёк»</t>
+          <t>ОДО «Северный Ветер»</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Аренда</t>
-        </is>
-      </c>
-      <c r="E31" t="inlineStr"/>
+          <t>Техническое обслуживание</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>27.09.2024</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>23.12.2024</t>
+        </is>
+      </c>
+      <c r="F31" t="n">
+        <v>35255</v>
+      </c>
+      <c r="G31" t="n">
+        <v>26441.25</v>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>На согласовании</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>АО «Одуванчик»</t>
+          <t>ООО «Гранит-Строй»</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Консультации</t>
-        </is>
-      </c>
-      <c r="D32" t="n">
-        <v>135000</v>
+          <t>Аренда помещения</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>28.01.2024</t>
+        </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>на подписании</t>
+          <t>26.12.2024</t>
+        </is>
+      </c>
+      <c r="F32" t="n">
+        <v>36600</v>
+      </c>
+      <c r="G32" t="n">
+        <v>36600</v>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>Завершён</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>ООО «Клевер»</t>
+          <t>ООО «Ромашка»</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Подряд</t>
-        </is>
-      </c>
-      <c r="D33" t="n">
-        <v>136250</v>
+          <t>Консультационные услуги</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>01.02.2024</t>
+        </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>закрыт</t>
-        </is>
+          <t>01.12.2024</t>
+        </is>
+      </c>
+      <c r="F33" t="n">
+        <v>36440</v>
+      </c>
+      <c r="G33" t="n">
+        <v>9110</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>ООО «Ромашка»</t>
+          <t>ИП Иванов И. И.</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Сопровождение</t>
-        </is>
-      </c>
-      <c r="D34" t="n">
-        <v>137500</v>
+          <t>Подряд на монтаж</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>02.03.2024</t>
+        </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>действует</t>
+          <t>04.12.2024</t>
+        </is>
+      </c>
+      <c r="F34" t="n">
+        <v>37785</v>
+      </c>
+      <c r="G34" t="n">
+        <v>18892.5</v>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>Расторгнут</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>ИП Иванов И. И.</t>
+          <t>ООО «Василёк»</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Поставка</t>
-        </is>
-      </c>
-      <c r="D35" t="n">
-        <v>138750</v>
-      </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>продлён</t>
+          <t>Оказание услуг</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>03.04.2024</t>
+        </is>
+      </c>
+      <c r="F35" t="n">
+        <v>39130</v>
+      </c>
+      <c r="G35" t="n">
+        <v>29347.5</v>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>Действует</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>ООО «Василёк»</t>
+          <t>ЗАО «Тестовый Мост»</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Аренда</t>
-        </is>
-      </c>
-      <c r="D36" t="n">
-        <v>140000</v>
-      </c>
-      <c r="E36" t="inlineStr"/>
+          <t>Поставка оборудования</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>04.05.2024</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>10.12.2024</t>
+        </is>
+      </c>
+      <c r="F36" t="n">
+        <v>40475</v>
+      </c>
+      <c r="G36" t="n">
+        <v>40475</v>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>На согласовании</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>АО «Одуванчик»</t>
+          <t>ООО «ТехноСфера-Плюс»</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Консультации</t>
-        </is>
-      </c>
-      <c r="D37" t="n">
-        <v>141250</v>
+          <t>Техническое обслуживание</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>05.06.2024</t>
+        </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>на подписании</t>
+          <t>13.12.2024</t>
+        </is>
+      </c>
+      <c r="F37" t="n">
+        <v>41820</v>
+      </c>
+      <c r="G37" t="n">
+        <v>10455</v>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>Завершён</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>ООО «Клевер»</t>
+          <t>ОДО «Северный Ветер»</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Подряд</t>
+          <t>Аренда помещения</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>06.07.2024</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>закрыт</t>
+          <t>16.12.2024</t>
+        </is>
+      </c>
+      <c r="F38" t="n">
+        <v>43165</v>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>Продлён</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>ООО «Ромашка»</t>
+          <t>ООО «Гранит-Строй»</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Сопровождение</t>
-        </is>
-      </c>
-      <c r="D39" t="n">
-        <v>143750</v>
+          <t>Консультационные услуги</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>07.08.2024</t>
+        </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>действует</t>
+          <t>19.12.2024</t>
+        </is>
+      </c>
+      <c r="F39" t="n">
+        <v>44510</v>
+      </c>
+      <c r="G39" t="n">
+        <v>33382.5</v>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>Расторгнут</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>ИП Иванов И. И.</t>
+          <t>ООО «Ромашка»</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Поставка</t>
-        </is>
-      </c>
-      <c r="D40" t="n">
-        <v>145000</v>
-      </c>
-      <c r="E40" t="inlineStr">
-        <is>
-          <t>продлён</t>
-        </is>
+          <t>Подряд на монтаж</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>08.09.2024</t>
+        </is>
+      </c>
+      <c r="F40" t="n">
+        <v>44350</v>
+      </c>
+      <c r="G40" t="n">
+        <v>44350</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>ООО «Василёк»</t>
+          <t>ИП Иванов И. И.</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Аренда</t>
-        </is>
-      </c>
-      <c r="D41" t="n">
-        <v>146250</v>
-      </c>
-      <c r="E41" t="inlineStr"/>
+          <t>Оказание услуг</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>09.01.2024</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>25.12.2024</t>
+        </is>
+      </c>
+      <c r="F41" t="n">
+        <v>45695</v>
+      </c>
+      <c r="G41" t="n">
+        <v>11423.75</v>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>На согласовании</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>АО «Одуванчик»</t>
+          <t>ООО «Василёк»</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Консультации</t>
-        </is>
-      </c>
-      <c r="D42" t="n">
-        <v>147500</v>
+          <t>Поставка оборудования</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>10.02.2024</t>
+        </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>на подписании</t>
+          <t>28.12.2024</t>
+        </is>
+      </c>
+      <c r="F42" t="n">
+        <v>47040</v>
+      </c>
+      <c r="G42" t="n">
+        <v>23520</v>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Завершён</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
+        <v>39</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>ЗАО «Тестовый Мост»</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Техническое обслуживание</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>11.03.2024</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>03.12.2024</t>
+        </is>
+      </c>
+      <c r="F43" t="n">
+        <v>48385</v>
+      </c>
+      <c r="G43" t="n">
+        <v>36288.75</v>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>Продлён</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
         <v>40</v>
       </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>ООО «Клевер»</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>Подряд</t>
-        </is>
-      </c>
-      <c r="D43" t="n">
-        <v>148750</v>
-      </c>
-      <c r="E43" t="inlineStr">
-        <is>
-          <t>закрыт</t>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>ООО «ТехноСфера-Плюс»</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Аренда помещения</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>12.04.2024</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>06.12.2024</t>
+        </is>
+      </c>
+      <c r="F44" t="n">
+        <v>49730</v>
+      </c>
+      <c r="G44" t="n">
+        <v>49730</v>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>Расторгнут</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="B45" t="inlineStr">
+      <c r="A45" s="3" t="inlineStr">
         <is>
           <t>Итого</t>
         </is>
       </c>
-      <c r="D45">
-        <f>SUM(D4:D43)</f>
-        <v/>
+      <c r="F45" s="4" t="n">
+        <v>1098125</v>
+      </c>
+      <c r="G45" s="4" t="n">
+        <v>637416.25</v>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="B45:C45"/>
+  <mergeCells count="8">
+    <mergeCell ref="F3:G3"/>
+    <mergeCell ref="C3:C4"/>
+    <mergeCell ref="B3:B4"/>
+    <mergeCell ref="A3:A4"/>
+    <mergeCell ref="H3:H4"/>
+    <mergeCell ref="A45:E45"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="D3:E3"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1351,61 +1914,151 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Показатель</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Значение</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Ставка НДС</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>0.2</v>
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>Сводка по кварталам</t>
+        </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Сумма без НДС</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>250000</v>
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Квартал</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>План, BYN</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Факт, BYN</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>Отклонение</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>Признак</t>
+        </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>НДС</t>
-        </is>
-      </c>
-      <c r="B4">
-        <f>B3*B2</f>
+          <t>1 квартал</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>60000</v>
+      </c>
+      <c r="C4" t="n">
+        <v>58430.5</v>
+      </c>
+      <c r="D4">
+        <f>C4-B4</f>
+        <v>-1569.5</v>
+      </c>
+      <c r="E4">
+        <f>IF(C4&gt;=B4,"выполнен","не выполнен")</f>
         <v/>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Итого с НДС</t>
-        </is>
-      </c>
-      <c r="B5">
-        <f>B3+B4</f>
+          <t>2 квартал</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>72000</v>
+      </c>
+      <c r="C5" t="n">
+        <v>75120</v>
+      </c>
+      <c r="D5">
+        <f>C5-B5</f>
+        <v>3120</v>
+      </c>
+      <c r="E5">
+        <f>IF(C5&gt;=B5,"выполнен","не выполнен")</f>
         <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>3 квартал</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>65000</v>
+      </c>
+      <c r="C6" t="n">
+        <v>61004.25</v>
+      </c>
+      <c r="D6">
+        <f>C6-B6</f>
+        <v>-3995.75</v>
+      </c>
+      <c r="E6">
+        <f>IF(C6&gt;=B6,"выполнен","не выполнен")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>4 квартал</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>80000</v>
+      </c>
+      <c r="C7" t="n">
+        <v>79880.75</v>
+      </c>
+      <c r="D7">
+        <f>C7-B7</f>
+        <v>-119.25</v>
+      </c>
+      <c r="E7">
+        <f>IF(C7&gt;=B7,"выполнен","не выполнен")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Итого</t>
+        </is>
+      </c>
+      <c r="B8">
+        <f>SUM(B4:B7)</f>
+        <v>277000</v>
+      </c>
+      <c r="C8">
+        <f>SUM(C4:C7)</f>
+        <v>274435.5</v>
+      </c>
+      <c r="D8">
+        <f>SUM(D4:D7)</f>
+        <v>-2564.5</v>
       </c>
     </row>
   </sheetData>
@@ -1419,13 +2072,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="B2:B2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Лист оставлен почти пустым намеренно.</t>
+    <row r="2">
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Лист намеренно оставлен почти пустым.</t>
         </is>
       </c>
     </row>

</xml_diff>